<commit_message>
latest updated BE code
</commit_message>
<xml_diff>
--- a/excel/2026/August/UG_Admissions.xlsx
+++ b/excel/2026/August/UG_Admissions.xlsx
@@ -479,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" style="1" customWidth="1"/>
@@ -567,6 +567,9 @@
     <row r="3" ht="20" customHeight="1" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="20" customHeight="1" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="5" ht="20" customHeight="1" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="20" customHeight="1" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="20" customHeight="1" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="8" ht="20" customHeight="1" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>